<commit_message>
Replace files as i moved the screw terminal on the JST version of the PCB
</commit_message>
<xml_diff>
--- a/PCB/JST/Fabrication/PickAndPlace_PCB_JST.xlsx
+++ b/PCB/JST/Fabrication/PickAndPlace_PCB_JST.xlsx
@@ -160,13 +160,13 @@
     <t>CONN-TH_2P-P5.00_WJ500V-5.08-2P</t>
   </si>
   <si>
-    <t>56.858mm</t>
-  </si>
-  <si>
-    <t>-6.151mm</t>
-  </si>
-  <si>
-    <t>54.318mm</t>
+    <t>57.023mm</t>
+  </si>
+  <si>
+    <t>-5.588mm</t>
+  </si>
+  <si>
+    <t>54.483mm</t>
   </si>
   <si>
     <t>No</t>

</xml_diff>

<commit_message>
reuploaded all of the files for the JST version as i moved the reset button + Update Journal.md
</commit_message>
<xml_diff>
--- a/PCB/JST/Fabrication/PickAndPlace_PCB_JST.xlsx
+++ b/PCB/JST/Fabrication/PickAndPlace_PCB_JST.xlsx
@@ -346,13 +346,13 @@
     <t>SW-SMD_L3.9-W3.0-P4.45</t>
   </si>
   <si>
-    <t>3.429mm</t>
-  </si>
-  <si>
-    <t>-6.223mm</t>
-  </si>
-  <si>
-    <t>5.614mm</t>
+    <t>12.853mm</t>
+  </si>
+  <si>
+    <t>-9.932mm</t>
+  </si>
+  <si>
+    <t>-7.747mm</t>
   </si>
   <si>
     <t>SW2</t>
@@ -1975,10 +1975,10 @@
         <v>112</v>
       </c>
       <c r="H17" t="s">
+        <v>111</v>
+      </c>
+      <c r="I17" t="s">
         <v>113</v>
-      </c>
-      <c r="I17" t="s">
-        <v>112</v>
       </c>
       <c r="J17">
         <v>2</v>
@@ -1987,7 +1987,7 @@
         <v>21</v>
       </c>
       <c r="L17">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="M17" t="s">
         <v>22</v>

</xml_diff>